<commit_message>
Update with new GX lot
</commit_message>
<xml_diff>
--- a/gx_lotmapping/std_curve_params.xlsx
+++ b/gx_lotmapping/std_curve_params.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yjin\Documents\projects\GeneXpert_WW\gx_lotmapping\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nhizon\Desktop\GeneXpert_WW\gx_lotmapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="59">
   <si>
     <t>Cartridge Lot Number</t>
   </si>
@@ -1056,7 +1056,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
@@ -2346,32 +2346,32 @@
         <v>11</v>
       </c>
     </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65">
+        <v>49312</v>
+      </c>
+      <c r="B65" t="s">
+        <v>26</v>
+      </c>
+      <c r="C65" t="s">
+        <v>8</v>
+      </c>
+      <c r="D65" t="s">
+        <v>9</v>
+      </c>
+      <c r="E65" t="s">
+        <v>10</v>
+      </c>
+      <c r="F65" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4ab521e1-8720-4533-8025-5c945dd49c24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="16e82f90-a588-4221-9ba0-cc9a2dc4dcab" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC70BFA850CCAE47A7BAA0F38D9D36E7" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca04f000950caa8121282a10b5ee4284">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4ab521e1-8720-4533-8025-5c945dd49c24" xmlns:ns3="16e82f90-a588-4221-9ba0-cc9a2dc4dcab" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a7a7c827840bdaa11f304efd419307b4" ns2:_="" ns3:_="">
     <xsd:import namespace="4ab521e1-8720-4533-8025-5c945dd49c24"/>
@@ -2600,26 +2600,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBC8AA1D-4A1F-4E6B-AEE1-0D75C632111C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4ab521e1-8720-4533-8025-5c945dd49c24"/>
-    <ds:schemaRef ds:uri="16e82f90-a588-4221-9ba0-cc9a2dc4dcab"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3305E1E3-DAA1-4965-97DA-EEFD152C6338}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4ab521e1-8720-4533-8025-5c945dd49c24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="16e82f90-a588-4221-9ba0-cc9a2dc4dcab" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1557CBC2-664F-4BAE-96F8-E7372F324347}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2636,4 +2637,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3305E1E3-DAA1-4965-97DA-EEFD152C6338}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBC8AA1D-4A1F-4E6B-AEE1-0D75C632111C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4ab521e1-8720-4533-8025-5c945dd49c24"/>
+    <ds:schemaRef ds:uri="16e82f90-a588-4221-9ba0-cc9a2dc4dcab"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added 60622 gx lot
</commit_message>
<xml_diff>
--- a/gx_lotmapping/std_curve_params.xlsx
+++ b/gx_lotmapping/std_curve_params.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nhizon\Desktop\GeneXpert_WW\gx_lotmapping\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yjin\Documents\projects\GeneXpert_WW\gx_lotmapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="59">
   <si>
     <t>Cartridge Lot Number</t>
   </si>
@@ -1056,7 +1056,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
@@ -2347,7 +2347,7 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65">
+      <c r="A65" s="3">
         <v>49312</v>
       </c>
       <c r="B65" t="s">
@@ -2363,6 +2363,26 @@
         <v>10</v>
       </c>
       <c r="F65" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="3">
+        <v>60622</v>
+      </c>
+      <c r="B66" t="s">
+        <v>26</v>
+      </c>
+      <c r="C66" t="s">
+        <v>8</v>
+      </c>
+      <c r="D66" t="s">
+        <v>9</v>
+      </c>
+      <c r="E66" t="s">
+        <v>10</v>
+      </c>
+      <c r="F66" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2601,15 +2621,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="4ab521e1-8720-4533-8025-5c945dd49c24">
@@ -2618,6 +2629,15 @@
     <TaxCatchAll xmlns="16e82f90-a588-4221-9ba0-cc9a2dc4dcab" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2640,14 +2660,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3305E1E3-DAA1-4965-97DA-EEFD152C6338}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBC8AA1D-4A1F-4E6B-AEE1-0D75C632111C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2656,4 +2668,12 @@
     <ds:schemaRef ds:uri="16e82f90-a588-4221-9ba0-cc9a2dc4dcab"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3305E1E3-DAA1-4965-97DA-EEFD152C6338}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added GX lot 62905
</commit_message>
<xml_diff>
--- a/gx_lotmapping/std_curve_params.xlsx
+++ b/gx_lotmapping/std_curve_params.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yjin\Documents\projects\GeneXpert_WW\gx_lotmapping\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nhizon\Desktop\GeneXpert_WW\gx_lotmapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="59">
   <si>
     <t>Cartridge Lot Number</t>
   </si>
@@ -1056,7 +1056,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
@@ -2386,12 +2386,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="3">
+        <v>62905</v>
+      </c>
+      <c r="B67" t="s">
+        <v>26</v>
+      </c>
+      <c r="C67" t="s">
+        <v>8</v>
+      </c>
+      <c r="D67" t="s">
+        <v>9</v>
+      </c>
+      <c r="E67" t="s">
+        <v>10</v>
+      </c>
+      <c r="F67" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4ab521e1-8720-4533-8025-5c945dd49c24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="16e82f90-a588-4221-9ba0-cc9a2dc4dcab" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC70BFA850CCAE47A7BAA0F38D9D36E7" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca04f000950caa8121282a10b5ee4284">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4ab521e1-8720-4533-8025-5c945dd49c24" xmlns:ns3="16e82f90-a588-4221-9ba0-cc9a2dc4dcab" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a7a7c827840bdaa11f304efd419307b4" ns2:_="" ns3:_="">
     <xsd:import namespace="4ab521e1-8720-4533-8025-5c945dd49c24"/>
@@ -2620,27 +2660,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4ab521e1-8720-4533-8025-5c945dd49c24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="16e82f90-a588-4221-9ba0-cc9a2dc4dcab" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3305E1E3-DAA1-4965-97DA-EEFD152C6338}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBC8AA1D-4A1F-4E6B-AEE1-0D75C632111C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4ab521e1-8720-4533-8025-5c945dd49c24"/>
+    <ds:schemaRef ds:uri="16e82f90-a588-4221-9ba0-cc9a2dc4dcab"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1557CBC2-664F-4BAE-96F8-E7372F324347}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2657,23 +2696,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBC8AA1D-4A1F-4E6B-AEE1-0D75C632111C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4ab521e1-8720-4533-8025-5c945dd49c24"/>
-    <ds:schemaRef ds:uri="16e82f90-a588-4221-9ba0-cc9a2dc4dcab"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3305E1E3-DAA1-4965-97DA-EEFD152C6338}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>